<commit_message>
M4: Scopus enrichment with fallbacks and offline mock
- ScopusService: FULL-view retrieval by EID then DOI, request throttling,
  X-RateLimit-aware pausing, tenacity backoff honoring Retry-After, and
  auth failures that disable the provider without failing individual rows
- Tolerant JSON walkers (_dig/_as_list/_unwrap) for Elsevier's collapsed
  single-element arrays, {"$": ...} wrappers, and the two abstract locations
- Semantic Scholar and Crossref fallbacks; Crossref never supplies abstracts
  so metadata-only rows stay INCOMPLETE rather than fabricating support
- MockScopusService runs fixture payloads through the real parser
- Fixtures now withhold three abstracts so enrichment is genuinely exercised

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample_dataset.xlsx
+++ b/tests/fixtures/sample_dataset.xlsx
@@ -624,11 +624,7 @@
           <t>https://doi.org/10.1016/j.knosys.2021.100004</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Fraudulent transactions represent a tiny fraction of payment traffic, which makes anomaly detectors prone to majority-class bias. We compare resampling, cost-sensitive learning, and synthetic minority oversampling, and report that cost-sensitive objectives give the most stable precision-recall trade-off in production settings.</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>class imbalance; anomaly detection; SMOTE</t>
@@ -710,11 +706,7 @@
           <t>https://doi.org/10.1109/ACCESS.2020.100006</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Payment systems form dense transaction graphs whose structure carries signal about coordinated abuse. We apply graph neural networks to inter-account transfer graphs and detect collusive rings that node-level classifiers miss entirely.</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>graph neural networks; payment networks; collusion</t>
@@ -839,11 +831,7 @@
           <t>https://doi.org/10.1016/j.patrec.2021.100009</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Accuracy is misleading when the positive class is rare. We formalise the relationship between precision-recall area and cost-weighted utility, and recommend reporting partial AUC at operationally relevant false positive rates.</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>evaluation metrics; imbalanced data; precision-recall</t>

</xml_diff>